<commit_message>
refactor: update database initialization and similarity matrix calculation
</commit_message>
<xml_diff>
--- a/data/raw/english-japanese-raw-parallel.xlsx
+++ b/data/raw/english-japanese-raw-parallel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dolph\Projects\2026-NLP-Project\Cross-Language-Distance-Visualizer\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3423544-BE72-4AE5-8F5A-1FD73A94AEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{250606C8-ED56-4E8E-9B51-3AD9B435ADF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3340" yWindow="3340" windowWidth="16800" windowHeight="9670" xr2:uid="{AADE9F91-D15F-4FD3-84BB-1315A195BAF2}"/>
   </bookViews>
@@ -41,15 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="130">
   <si>
-    <t>English</t>
-  </si>
-  <si>
-    <t>Japanese</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Which team do you support?</t>
   </si>
   <si>
@@ -429,6 +420,15 @@
   </si>
   <si>
     <t>あなたと話がしたいなぁ。</t>
+  </si>
+  <si>
+    <t>english</t>
+  </si>
+  <si>
+    <t>japanese</t>
+  </si>
+  <si>
+    <t>type</t>
   </si>
 </sst>
 </file>
@@ -809,695 +809,695 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>127</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>128</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C17" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B19" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C23" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C24" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C25" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B28" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C28" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C29" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B30" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C30" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B31" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C31" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C32" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C33" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B34" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C34" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B35" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C35" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C36" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B37" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C37" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C38" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C39" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C40" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C41" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B42" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C42" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B43" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C43" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C44" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C45" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C46" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C47" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C48" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C49" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B50" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C50" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B51" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C51" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B52" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C52" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B53" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C53" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B54" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C54" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C55" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B56" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C56" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B57" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C57" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B58" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C58" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B59" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C59" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B60" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C60" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B61" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C61" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B62" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C62" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B63" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C63" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1506,15 +1506,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA54F7F47019384D918F48D02CD9E8C0" ma:contentTypeVersion="8" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2fd060fc4a81960741b3e3329c9ee275">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2c7252f8-1396-4cde-9d89-c4eb695c0555" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1386d2417a839c3f2ba3e30e582258f8" ns3:_="">
     <xsd:import namespace="2c7252f8-1396-4cde-9d89-c4eb695c0555"/>
@@ -1682,6 +1673,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1691,14 +1691,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60A2657-49AE-4A6D-906F-9E2B07D050C1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0FB1AA0-A3E1-4C08-8982-7ABB3DB69A0E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1712,6 +1704,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F60A2657-49AE-4A6D-906F-9E2B07D050C1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>